<commit_message>
Save library recording Session 12/10/2026, 01:28:15 - 59188e01-2be0-460a-b044-f78738d1f6ef - 2026-10-11T14:34:31.267300Z
</commit_message>
<xml_diff>
--- a/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/59188e01-2be0-460a-b044-f78738d1f6ef/resources/azure-devops.xlsx
+++ b/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/59188e01-2be0-460a-b044-f78738d1f6ef/resources/azure-devops.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,797 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open https://hfm-wholesale-app-dev.ashysand-8cabb4df.australiaeast.azurecontainerapps.io/daily-orders?storeNo=426&amp;date=2026-10-08</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://hfm-wholesale-app-dev.ashysand-8cabb4df.australiaeast.azurecontainerapps.io/daily-orders?storeNo=426&amp;date=2026-10-08</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Click 126,319</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)", "x": 126, "y": 319, "text": "", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>step-002.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Type: Sa</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sa</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)"}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>step-003.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Click 136,411</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)", "x": 136, "y": 411, "text": "", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>step-004.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Type: {{HFM_Ext_pass}}</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>{{HFM_Ext_pass}}</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)"}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>step-005.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Click Sign in</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{"primary": "#root &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; button:nth-of-type(1)", "x": 306, "y": 505, "text": "Sign in", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>step-006.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Click HFM Internal Production</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"primary": "main:nth-of-type(1) &gt; section:nth-of-type(1) &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; select:nth-of-type(1)", "x": 146, "y": 242, "text": "HFM Internal Production", "tag": "select"}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>step-007.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Type: Hi tech</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Hi tech</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{"primary": "input[placeholder=\"Search stores\"]"}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>step-008.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Click HFM Internal Production</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{"primary": "main:nth-of-type(1) &gt; section:nth-of-type(1) &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; select:nth-of-type(1)", "x": 220, "y": 263, "text": "HFM Internal Production", "tag": "select"}</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>step-009.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Click HFM Internal Production</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{"primary": "main:nth-of-type(1) &gt; section:nth-of-type(1) &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; select:nth-of-type(1)", "x": 215, "y": 260, "text": "HFM Internal Production", "tag": "select"}</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>step-010.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Click Filter stores</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{"primary": "input[aria-label=\"Filter stores\"]", "x": 293, "y": 318, "text": "Filter stores", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>step-011.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Type: Tech</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{"primary": "input[placeholder=\"Search stores\"]"}</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>step-012.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Click Hi-Tech
+Store 426</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{"primary": "#\\:r2\\: &gt; button:nth-of-type(1)", "x": 212, "y": 378, "text": "Hi-Tech\nStore 426", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>step-013.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Click Monday 19th of October 2026
+Friday 16th of October 2026
+Thursday 15th of October</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; main:nth-of-type(1) &gt; section:nth-of-type(1) &gt; div:nth-of-type(3) &gt; label:nth-of-type(1) &gt; select:nth-of-type(1)", "x": 500, "y": 245, "text": "Monday 19th of October 2026\nFriday 16th of October 2026\nThursday 15th of October", "tag": "select"}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>step-014.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Click ASIAN - BABY / SHANGHI BOK CHOY</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{"primary": "section:nth-of-type(1) &gt; div:nth-of-type(4) &gt; table:nth-of-type(1) &gt; tbody:nth-of-type(1) &gt; tr:nth-of-type(1) &gt; td:nth-of-type(4)", "x": 437, "y": 404, "text": "ASIAN - BABY / SHANGHI BOK CHOY", "tag": "td"}</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>step-015.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Click Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY\"]", "x": 675, "y": 412, "text": "Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>step-016.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Type: 5</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(4) &gt; table:nth-of-type(1) &gt; tbody:nth-of-type(1) &gt; tr:nth-of-type(1) &gt; td:nth-of-type(6) &gt; input:nth-of-type(1)"}</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>step-017.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Press Enter</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Enter</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>step-018.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Click 657,475</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>{"primary": "section:nth-of-type(1) &gt; div:nth-of-type(4) &gt; table:nth-of-type(1) &gt; tbody:nth-of-type(1) &gt; tr:nth-of-type(2) &gt; td:nth-of-type(6)", "x": 657, "y": 475, "text": "", "tag": "td"}</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>step-019.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Type: 2</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>step-020.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Click Ordered quantity for ASIAN - BUK CHOY - EACH</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - BUK CHOY - EACH\"]", "x": 675, "y": 449, "text": "Ordered quantity for ASIAN - BUK CHOY - EACH", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>step-021.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Click Ordered quantity for ASIAN - CHOY SUM - EACH</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - CHOY SUM - EACH\"]", "x": 685, "y": 517, "text": "Ordered quantity for ASIAN - CHOY SUM - EACH", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>step-022.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Click Ordered quantity for ASIAN - CHOY SUM - EACH</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - CHOY SUM - EACH\"]", "x": 688, "y": 504, "text": "Ordered quantity for ASIAN - CHOY SUM - EACH", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>step-023.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Click Comment for ASIAN - BUK CHOY - EACH</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>{"primary": "input[aria-label=\"Comment for ASIAN - BUK CHOY - EACH\"]", "x": 874, "y": 464, "text": "Comment for ASIAN - BUK CHOY - EACH", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>step-024.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Type: Test automation tool</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Test automation tool</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(4) &gt; table:nth-of-type(1) &gt; tbody:nth-of-type(1) &gt; tr:nth-of-type(2) &gt; td:nth-of-type(8) &gt; input:nth-of-type(1)"}</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>step-025.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Click 753,538</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>{"primary": "#\\:r0\\:-1152\\%7C10012-shipped", "x": 753, "y": 538, "text": "", "tag": "td"}</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>step-026.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 01:28:15</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Click Sign out</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>{"primary": "#root &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; header:nth-of-type(1) &gt; div:nth-of-type(2) &gt; button:nth-of-type(1)", "x": 971, "y": 31, "text": "Sign out", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>step-027.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>